<commit_message>
Retrait du kit feu vert DSI : pile, FAQ, carte des heures perdues et documents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LC4TupPrFso4836h2aRcwR
</commit_message>
<xml_diff>
--- a/bonus/2026-10-12_carte-des-heures-perdues.xlsx
+++ b/bonus/2026-10-12_carte-des-heures-perdues.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mode d’emploi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Paramètres" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Listes" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="Équipe" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Saisie" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Synthèse" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d’emploi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paramètres" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Équipe" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saisie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -637,7 +637,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>4. Envoyez avec le tableur deux documents types par tâche, anonymisés avec la fiche du kit feu vert DSI.</t>
+          <t>4. Envoyez avec le tableur deux documents types par tâche, anonymisés : chaque nom est remplacé par un repère entre crochets, comme [CLIENT A].</t>
         </is>
       </c>
     </row>

</xml_diff>